<commit_message>
Actualiza cronograma de actividades
</commit_message>
<xml_diff>
--- a/cronogramas de actividades.xlsx
+++ b/cronogramas de actividades.xlsx
@@ -1,50 +1,69 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FabricioAlexanderBor\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE9B0F0-FB61-41DE-A376-0F7F8438A073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A27F3596-AB50-450F-A67D-74E0875C2200}"/>
+    <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet r:id="rId1" name="Hoja1" sheetId="1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0" iterateCount="100" iterateDelta="0.001"/>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+  <si>
+    <t>CRONOGRAMA DE ACTIVIDADES DE TICS</t>
+  </si>
   <si>
     <t>NOMBRE DEL PROYECTO:</t>
   </si>
   <si>
+    <t xml:space="preserve">Sistema Informatico de Gestión </t>
+  </si>
+  <si>
     <t>ÁREA  REQUIRIENTE:</t>
   </si>
   <si>
+    <t>Academica</t>
+  </si>
+  <si>
     <t>USUARIO QUE SOLICITA:</t>
   </si>
   <si>
+    <t>Hector Lopez</t>
+  </si>
+  <si>
+    <t>RESPONSABLE DEL DESARROLLO</t>
+  </si>
+  <si>
+    <t>Fabricio Borja</t>
+  </si>
+  <si>
     <t>NOMBRE DEL MÓDULO</t>
   </si>
   <si>
@@ -54,33 +73,15 @@
     <t>FECHA INICO</t>
   </si>
   <si>
+    <t>FECHA ENTREGA</t>
+  </si>
+  <si>
     <t>No. DE DÍAS</t>
   </si>
   <si>
     <t>OBSERVACIONES</t>
   </si>
   <si>
-    <t>FECHA ENTREGA</t>
-  </si>
-  <si>
-    <t>RESPONSABLE DEL DESARROLLO</t>
-  </si>
-  <si>
-    <t>CRONOGRAMA DE ACTIVIDADES DE TICS</t>
-  </si>
-  <si>
-    <t>Academica</t>
-  </si>
-  <si>
-    <t>Hector Lopez</t>
-  </si>
-  <si>
-    <t>Fabricio Borja</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sistema Informatico de Gestión </t>
-  </si>
-  <si>
     <t>PB-01 | Inicio de sesión</t>
   </si>
   <si>
@@ -111,6 +112,9 @@
     <t>PB-04 | Asignación de roles</t>
   </si>
   <si>
+    <t>Asignación y modificación de roles: administrador, responsable(Basado en cada areapor jerarquia), evaluador y consultor.</t>
+  </si>
+  <si>
     <t>Gestión de roles | Sprint 1 | Alta | Dep.: PB-03</t>
   </si>
   <si>
@@ -331,9 +335,6 @@
   </si>
   <si>
     <t>Desde 10/04/2026 hasta 20/07/2026</t>
-  </si>
-  <si>
-    <t>Asignación y modificación de roles: administrador, responsable(Basado en cada areapor jerarquia), evaluador y consultor.</t>
   </si>
   <si>
     <t xml:space="preserve"> </t>
@@ -342,40 +343,41 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="171" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
+      <b val="0"/>
+      <i val="0"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <i val="0"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <i val="0"/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <i val="0"/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -388,8 +390,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="8" tint="0.4"/>
       </patternFill>
     </fill>
   </fills>
@@ -403,29 +404,29 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </left>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -433,90 +434,99 @@
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="1" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+  <bag type="DXFComplements" extRef="DXFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -562,7 +572,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -614,7 +624,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -666,7 +676,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -675,816 +685,840 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7C9B227-0DFA-4004-A59F-E519184C52CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{233D0204-E7EE-457D-8ECC-17DB6AB60119}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K37"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="23.7109375" customWidth="1"/>
-    <col min="2" max="2" width="36.28515625" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.28125" customWidth="1"/>
+    <col min="3" max="3" width="13.00390625" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="32.57421875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="2"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="2"/>
-    </row>
-    <row r="3" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="7" t="s">
+      <c r="C8" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="9"/>
-    </row>
-    <row r="4" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-    </row>
-    <row r="6" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="4"/>
-      <c r="C6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+    </row>
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="11">
         <v>46122</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="11">
         <v>46125</v>
       </c>
       <c r="E9" s="12">
         <v>2</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="10" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="11">
         <v>46126</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="11">
         <v>46126</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="11">
         <v>46127</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="11">
         <v>46128</v>
       </c>
       <c r="E11" s="12">
         <v>2</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="J11" s="3"/>
-    </row>
-    <row r="12" spans="1:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="J11" s="13"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="C12" s="14">
+      <c r="B12" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="11">
         <v>46129</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="11">
         <v>46132</v>
       </c>
       <c r="E12" s="12">
         <v>2</v>
       </c>
-      <c r="F12" s="15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
+      <c r="F12" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="15" t="s">
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="14">
+      <c r="B13" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="11">
         <v>46133</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="11">
         <v>46135</v>
       </c>
       <c r="E13" s="12">
         <v>3</v>
       </c>
-      <c r="F13" s="15" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="F13" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="15" t="s">
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="14">
+      <c r="B14" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="11">
         <v>46136</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="11">
         <v>46139</v>
       </c>
       <c r="E14" s="12">
         <v>2</v>
       </c>
-      <c r="F14" s="15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
+      <c r="F14" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="15" t="s">
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="14">
+      <c r="B15" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="11">
         <v>46140</v>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="11">
         <v>46141</v>
       </c>
       <c r="E15" s="12">
         <v>2</v>
       </c>
-      <c r="F15" s="15" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
+      <c r="F15" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B16" s="15" t="s">
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="14">
+      <c r="B16" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="11">
         <v>46142</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="11">
         <v>46143</v>
       </c>
       <c r="E16" s="12">
         <v>2</v>
       </c>
-      <c r="F16" s="15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
+      <c r="F16" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="15" t="s">
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="14">
+      <c r="B17" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="11">
         <v>46146</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="11">
         <v>46148</v>
       </c>
       <c r="E17" s="12">
         <v>3</v>
       </c>
-      <c r="F17" s="15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+      <c r="F17" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="15" t="s">
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="14">
+      <c r="B18" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="11">
         <v>46149</v>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" s="11">
         <v>46153</v>
       </c>
       <c r="E18" s="12">
         <v>3</v>
       </c>
-      <c r="F18" s="15" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
+      <c r="F18" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B19" s="15" t="s">
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="14">
+      <c r="B19" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="11">
         <v>46154</v>
       </c>
-      <c r="D19" s="14">
+      <c r="D19" s="11">
         <v>46155</v>
       </c>
       <c r="E19" s="12">
         <v>2</v>
       </c>
-      <c r="F19" s="15" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
+      <c r="F19" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="15" t="s">
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="14">
+      <c r="B20" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="11">
         <v>46156</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="11">
         <v>46162</v>
       </c>
       <c r="E20" s="12">
         <v>5</v>
       </c>
-      <c r="F20" s="15" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="F20" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="15" t="s">
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="14">
+      <c r="B21" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="11">
         <v>46163</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21" s="11">
         <v>46167</v>
       </c>
       <c r="E21" s="12">
         <v>3</v>
       </c>
-      <c r="F21" s="15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
+      <c r="F21" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="15" t="s">
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="14">
+      <c r="B22" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="11">
         <v>46168</v>
       </c>
-      <c r="D22" s="14">
+      <c r="D22" s="11">
         <v>46170</v>
       </c>
       <c r="E22" s="12">
         <v>3</v>
       </c>
-      <c r="F22" s="15" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
+      <c r="F22" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="B23" s="15" t="s">
+    </row>
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C23" s="14">
+      <c r="B23" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" s="11">
         <v>46171</v>
       </c>
-      <c r="D23" s="14">
+      <c r="D23" s="11">
         <v>46177</v>
       </c>
       <c r="E23" s="12">
         <v>5</v>
       </c>
-      <c r="F23" s="15" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="60" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+      <c r="F23" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="B24" s="15" t="s">
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C24" s="14">
+      <c r="B24" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="11">
         <v>46178</v>
       </c>
-      <c r="D24" s="14">
+      <c r="D24" s="11">
         <v>46181</v>
       </c>
       <c r="E24" s="12">
         <v>2</v>
       </c>
-      <c r="F24" s="15" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+      <c r="F24" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="15" t="s">
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C25" s="14">
+      <c r="B25" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C25" s="11">
         <v>46182</v>
       </c>
-      <c r="D25" s="14">
+      <c r="D25" s="11">
         <v>46183</v>
       </c>
       <c r="E25" s="12">
         <v>2</v>
       </c>
-      <c r="F25" s="15" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
+      <c r="F25" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="B26" s="15" t="s">
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C26" s="14">
+      <c r="B26" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C26" s="11">
         <v>46184</v>
       </c>
-      <c r="D26" s="14">
+      <c r="D26" s="11">
         <v>46188</v>
       </c>
       <c r="E26" s="12">
         <v>3</v>
       </c>
-      <c r="F26" s="15" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+      <c r="F26" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="15" t="s">
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C27" s="14">
+      <c r="B27" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C27" s="11">
         <v>46189</v>
       </c>
-      <c r="D27" s="14">
+      <c r="D27" s="11">
         <v>46190</v>
       </c>
       <c r="E27" s="12">
         <v>2</v>
       </c>
-      <c r="F27" s="15" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
+      <c r="F27" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B28" s="15" t="s">
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C28" s="14">
+      <c r="B28" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" s="11">
         <v>46191</v>
       </c>
-      <c r="D28" s="14">
+      <c r="D28" s="11">
         <v>46195</v>
       </c>
       <c r="E28" s="12">
         <v>3</v>
       </c>
-      <c r="F28" s="15" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
-        <v>73</v>
-      </c>
-      <c r="B29" s="15" t="s">
+      <c r="F28" s="10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C29" s="14">
+      <c r="B29" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C29" s="11">
         <v>46196</v>
       </c>
-      <c r="D29" s="14">
+      <c r="D29" s="11">
         <v>46198</v>
       </c>
       <c r="E29" s="12">
         <v>3</v>
       </c>
-      <c r="F29" s="15" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
+      <c r="F29" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="B30" s="15" t="s">
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C30" s="14">
+      <c r="B30" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="11">
         <v>46199</v>
       </c>
-      <c r="D30" s="14">
+      <c r="D30" s="11">
         <v>46203</v>
       </c>
       <c r="E30" s="12">
         <v>3</v>
       </c>
-      <c r="F30" s="15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
+      <c r="F30" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B31" s="15" t="s">
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C31" s="14">
+      <c r="B31" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C31" s="11">
         <v>46204</v>
       </c>
-      <c r="D31" s="14">
+      <c r="D31" s="11">
         <v>46205</v>
       </c>
       <c r="E31" s="12">
         <v>2</v>
       </c>
-      <c r="F31" s="15" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A32" s="13" t="s">
+      <c r="F31" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="B32" s="15" t="s">
+    </row>
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C32" s="14">
+      <c r="B32" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="C32" s="11">
         <v>46206</v>
       </c>
-      <c r="D32" s="14">
+      <c r="D32" s="11">
         <v>46210</v>
       </c>
       <c r="E32" s="12">
         <v>3</v>
       </c>
-      <c r="F32" s="15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A33" s="13" t="s">
+      <c r="F32" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="B33" s="15" t="s">
+    </row>
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="C33" s="14">
+      <c r="B33" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C33" s="11">
         <v>46211</v>
       </c>
-      <c r="D33" s="14">
+      <c r="D33" s="11">
         <v>46212</v>
       </c>
       <c r="E33" s="12">
         <v>2</v>
       </c>
-      <c r="F33" s="15" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A34" s="13" t="s">
+      <c r="F33" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="B34" s="15" t="s">
+    </row>
+    <row r="34" ht="45" customHeight="1">
+      <c r="A34" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C34" s="14">
+      <c r="B34" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="C34" s="11">
         <v>46213</v>
       </c>
-      <c r="D34" s="14">
+      <c r="D34" s="11">
         <v>46217</v>
       </c>
       <c r="E34" s="12">
         <v>3</v>
       </c>
-      <c r="F34" s="15" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A35" s="13" t="s">
+      <c r="F34" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B35" s="15" t="s">
+    </row>
+    <row r="35" ht="45" customHeight="1">
+      <c r="A35" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="C35" s="14">
+      <c r="B35" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="C35" s="11">
         <v>46218</v>
       </c>
-      <c r="D35" s="14">
+      <c r="D35" s="11">
         <v>46219</v>
       </c>
       <c r="E35" s="12">
         <v>2</v>
       </c>
-      <c r="F35" s="15" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A36" s="13" t="s">
+      <c r="F35" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="B36" s="15" t="s">
+    </row>
+    <row r="36" ht="60" customHeight="1">
+      <c r="A36" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C36" s="14">
+      <c r="B36" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="C36" s="11">
         <v>46220</v>
       </c>
-      <c r="D36" s="14">
+      <c r="D36" s="11">
         <v>46223</v>
       </c>
       <c r="E36" s="12">
         <v>2</v>
       </c>
-      <c r="F36" s="15" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
+      <c r="F36" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="B37" s="16"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="17"/>
-      <c r="E37" s="11">
+    </row>
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B37" s="14"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="8">
         <v>72</v>
       </c>
-      <c r="F37" s="11" t="s">
-        <v>98</v>
+      <c r="F37" s="8" t="s">
+        <v>99</v>
       </c>
       <c r="K37" t="s">
         <v>100</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells>
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:F6"/>
@@ -1496,7 +1530,13 @@
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="C5:F5"/>
   </mergeCells>
+  <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
+  </headerFooter>
+  <extLst/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
carga de evaluacion y procesos para pruebas
</commit_message>
<xml_diff>
--- a/cronogramas de actividades.xlsx
+++ b/cronogramas de actividades.xlsx
@@ -345,7 +345,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
-    <numFmt numFmtId="228" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="456" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -359,7 +359,7 @@
     <font>
       <b/>
       <i val="0"/>
-      <sz val="11"/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
@@ -375,7 +375,7 @@
     <font>
       <b/>
       <i val="0"/>
-      <sz val="14"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
@@ -400,21 +400,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -454,6 +439,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -461,12 +461,15 @@
   </cellStyleXfs>
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
@@ -477,27 +480,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="228" fontId="0" fillId="0" borderId="1" xfId="0">
+    <xf numFmtId="456" fontId="0" fillId="0" borderId="4" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="1"/>
@@ -849,7 +849,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{28E4B4FC-293D-40F5-B3EE-E8B95CD97313}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{AE7C3C38-0B8E-4208-B543-1380A3D5AD72}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:K37"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="9.140625" customHeight="1"/>
   <cols>

</xml_diff>